<commit_message>
Daily slate 2026-06-30 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-28.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-28.xlsx
@@ -526,16 +526,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>424</v>
+        <v>439</v>
       </c>
       <c r="E4" t="n">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="F4" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="G4" t="n">
-        <v>43.4</v>
+        <v>43.1</v>
       </c>
     </row>
     <row r="5">
@@ -610,16 +610,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>290</v>
+        <v>304</v>
       </c>
       <c r="E7" t="n">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="F7" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="G7" t="n">
-        <v>56.6</v>
+        <v>57.6</v>
       </c>
     </row>
     <row r="8">
@@ -726,16 +726,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1535</v>
+        <v>1598</v>
       </c>
       <c r="E11" t="n">
-        <v>895</v>
+        <v>926</v>
       </c>
       <c r="F11" t="n">
-        <v>640</v>
+        <v>672</v>
       </c>
       <c r="G11" t="n">
-        <v>58.3</v>
+        <v>57.9</v>
       </c>
     </row>
     <row r="12">
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="E12" t="n">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="F12" t="n">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="G12" t="n">
-        <v>55.6</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">
@@ -784,13 +784,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E13" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F13" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G13" t="n">
         <v>50</v>
@@ -813,16 +813,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>477</v>
+        <v>496</v>
       </c>
       <c r="E14" t="n">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F14" t="n">
-        <v>371</v>
+        <v>387</v>
       </c>
       <c r="G14" t="n">
-        <v>22.2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15">
@@ -842,16 +842,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>563</v>
+        <v>589</v>
       </c>
       <c r="E15" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F15" t="n">
-        <v>474</v>
+        <v>498</v>
       </c>
       <c r="G15" t="n">
-        <v>15.8</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="16">
@@ -871,16 +871,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>538</v>
+        <v>547</v>
       </c>
       <c r="E16" t="n">
         <v>72</v>
       </c>
       <c r="F16" t="n">
-        <v>466</v>
+        <v>475</v>
       </c>
       <c r="G16" t="n">
-        <v>13.4</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="17">
@@ -900,13 +900,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5691</v>
+        <v>5980</v>
       </c>
       <c r="E17" t="n">
-        <v>858</v>
+        <v>900</v>
       </c>
       <c r="F17" t="n">
-        <v>4833</v>
+        <v>5080</v>
       </c>
       <c r="G17" t="n">
         <v>15.1</v>
@@ -1522,46 +1522,46 @@
         <v>251</v>
       </c>
       <c r="D7" t="n">
-        <v>58.3</v>
+        <v>57.9</v>
       </c>
       <c r="E7" t="n">
-        <v>1535</v>
+        <v>1598</v>
       </c>
       <c r="F7" t="n">
-        <v>55.6</v>
+        <v>56</v>
       </c>
       <c r="G7" t="n">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="H7" t="n">
         <v>50</v>
       </c>
       <c r="I7" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="J7" t="n">
-        <v>22.2</v>
+        <v>22</v>
       </c>
       <c r="K7" t="n">
-        <v>477</v>
+        <v>496</v>
       </c>
       <c r="L7" t="n">
-        <v>15.8</v>
+        <v>15.4</v>
       </c>
       <c r="M7" t="n">
-        <v>563</v>
+        <v>589</v>
       </c>
       <c r="N7" t="n">
-        <v>13.4</v>
+        <v>13.2</v>
       </c>
       <c r="O7" t="n">
-        <v>538</v>
+        <v>547</v>
       </c>
       <c r="P7" t="n">
         <v>15.1</v>
       </c>
       <c r="Q7" t="n">
-        <v>5691</v>
+        <v>5980</v>
       </c>
       <c r="R7" t="n">
         <v>45.7</v>
@@ -1570,10 +1570,10 @@
         <v>46</v>
       </c>
       <c r="T7" t="n">
-        <v>43.4</v>
+        <v>43.1</v>
       </c>
       <c r="U7" t="n">
-        <v>424</v>
+        <v>439</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
@@ -1594,10 +1594,10 @@
         <v>4</v>
       </c>
       <c r="AD7" t="n">
-        <v>56.6</v>
+        <v>57.6</v>
       </c>
       <c r="AE7" t="n">
-        <v>290</v>
+        <v>304</v>
       </c>
       <c r="AF7" t="n">
         <v>55</v>

</xml_diff>